<commit_message>
fix(template): adjust row heights, freeze panes, and standardize filename to 外贸出厂底价表与智能核价模板.xlsx
</commit_message>
<xml_diff>
--- a/public/templates/外贸出厂底价表与智能核价模板_双表旗舰版.xlsx
+++ b/public/templates/外贸出厂底价表与智能核价模板_双表旗舰版.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="162">
   <si>
-    <t>【2026 外贸出厂底价表与智能核价模板 · Kelvin旗舰版】使用指南</t>
+    <t>【2026外贸出厂底价表与智能核价模板】使用指南</t>
   </si>
   <si>
     <t>💡 本地离线版与线上版 KelvinFlow (https://quote.kelvinflow.com) 采用 100% 相同数据架构。在此填写的全部数据，日后可直接无损上传，零学习成本。</t>
@@ -710,7 +710,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1245,7 +1245,7 @@
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="85" customWidth="1"/>
+    <col min="3" max="3" width="92" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
@@ -1254,13 +1254,13 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" ht="24" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" ht="30" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" ht="52" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" ht="52" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
@@ -1276,7 +1276,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="7" ht="52" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
@@ -1284,7 +1284,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="8" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="9" ht="75" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="10" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>12</v>
       </c>

</xml_diff>